<commit_message>
fix(roster): apply the uploaded workbook to the managed admin input
2026-10-29: Preserve the workbook uploaded in aa6443d and apply its new employee 010424 to admin/설치업체.xlsx. Verify the prior 978 rows are unchanged, retain the leading zero, and regenerate the 979-worker asset. Remove the duplicate root copy so the next manual workflow reads the update.
</commit_message>
<xml_diff>
--- a/admin/설치업체.xlsx
+++ b/admin/설치업체.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\박희정\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\박희정\Desktop\새 폴더 (2)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAAF3A37-B266-4646-A371-E4A90F4B3670}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A32E7CB7-967E-447F-B9B7-3BDEEFAFDA40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{1C197A9B-D71D-44EF-A255-C08B5B1AAF55}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1C197A9B-D71D-44EF-A255-C08B5B1AAF55}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3844" uniqueCount="1969">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7696" uniqueCount="1973">
   <si>
     <t>사번</t>
   </si>
@@ -6913,6 +6913,22 @@
   </si>
   <si>
     <t>010613</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>010424</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>박희정</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>서일대대학교</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>손발팀</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -6964,7 +6980,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -6979,6 +6995,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7314,7 +7333,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B353774F-8F83-4164-9E89-B01AFFCDA0DC}">
-  <dimension ref="A1:D979"/>
+  <dimension ref="A1:D980"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="10.09765625" bestFit="1" customWidth="1"/>
@@ -20885,6 +20904,20 @@
         <v>1967</v>
       </c>
     </row>
+    <row r="980" spans="1:4">
+      <c r="A980" s="5" t="s">
+        <v>1969</v>
+      </c>
+      <c r="B980" s="1" t="s">
+        <v>1970</v>
+      </c>
+      <c r="C980" s="1" t="s">
+        <v>1971</v>
+      </c>
+      <c r="D980" t="s">
+        <v>1972</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>